<commit_message>
fix power switch alignment
</commit_message>
<xml_diff>
--- a/PCB/Altuim/Project Outputs for klor1_4/BOM/Bill of Materials-klor1_4.xlsx
+++ b/PCB/Altuim/Project Outputs for klor1_4/BOM/Bill of Materials-klor1_4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahmed\Work\KLOR\PCB\Altuim\Project Outputs for klor1_4\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BEEB8B1-A777-4BDE-A3B5-29705A4C6084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{189C6C65-A358-4D68-BA97-1ADAAD7C5479}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1780" yWindow="1780" windowWidth="17760" windowHeight="8640" xr2:uid="{7BA5F41C-C1A2-4AF5-8D2D-F58E3DFDDDB9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{15F09536-7A19-4834-84AA-CFFA7CBCD681}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-klor1_4" sheetId="1" r:id="rId1"/>
@@ -158,7 +158,7 @@
     <t>PSW1, PSW2</t>
   </si>
   <si>
-    <t>MSK12C02_REVERSIBLE</t>
+    <t>SW_MSK12C02</t>
   </si>
   <si>
     <t>Slide Switches SPDT switch length: 8mm, switch width: 2.8mm</t>
@@ -674,7 +674,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6CD0E92-942B-4511-AD2F-BD4AAED6BF90}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFD45C7-F1DE-4BCA-90BC-2BCD61A74E2A}">
   <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>

<commit_message>
adding BOM for haptic circuit
</commit_message>
<xml_diff>
--- a/PCB/Altuim/Project Outputs for klor1_4/BOM/Bill of Materials-klor1_4.xlsx
+++ b/PCB/Altuim/Project Outputs for klor1_4/BOM/Bill of Materials-klor1_4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahmed\Work\KLOR\PCB\Altuim\Project Outputs for klor1_4\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE3E6094-65EF-47B7-9795-04F91847B31D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF53B3FE-E58F-4809-89DF-E655BB02E827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1C5A7FCA-A99B-47B8-A61A-FE86534B49E4}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{8F8EA070-2F4B-4877-A16D-FC4F2D8C15A9}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-klor1_4" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="92">
   <si>
     <t>Designator</t>
   </si>
@@ -65,6 +65,27 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>U4, U6</t>
+  </si>
+  <si>
+    <t>SMD-16_ELV1411A</t>
+  </si>
+  <si>
+    <t>11mm x 14mm Rectangular Linear Vibration Motor Model NFP-ELV1411A-A1</t>
+  </si>
+  <si>
+    <t>JLCPCB Assembly</t>
+  </si>
+  <si>
+    <t>ELV1411</t>
+  </si>
+  <si>
+    <t>LCSC</t>
+  </si>
+  <si>
+    <t>C9900029336</t>
+  </si>
+  <si>
     <t>SW1, SW2, SW3, SW4, SW5, SW6, SW7, SW8, SW9, SW10, SW11, SW12, SW13, SW14, SW15, SW16, SW17, SW19, SW20, SW21, SW22, SW23, SW24, SW25, SW26, SW27, SW28, SW29, SW30, SW31, SW32, SW33, SW34, SW35, SW36, SW37, SW38, SW39, SW40, SW41, SW42, SW43</t>
   </si>
   <si>
@@ -80,9 +101,6 @@
     <t>CPG151101S11-16</t>
   </si>
   <si>
-    <t>LCSC</t>
-  </si>
-  <si>
     <t>C41430893</t>
   </si>
   <si>
@@ -119,6 +137,21 @@
     <t>C5149201</t>
   </si>
   <si>
+    <t>C1, C2, C3, C4</t>
+  </si>
+  <si>
+    <t>FP-C0402-BB-MFG</t>
+  </si>
+  <si>
+    <t>CCTC</t>
+  </si>
+  <si>
+    <t>TCC0402X5R105M100AT</t>
+  </si>
+  <si>
+    <t>C2887020</t>
+  </si>
+  <si>
     <t>SW18, SW44</t>
   </si>
   <si>
@@ -173,6 +206,24 @@
     <t>C431540</t>
   </si>
   <si>
+    <t>U3, U5</t>
+  </si>
+  <si>
+    <t>FP-DGS0010A-MFG</t>
+  </si>
+  <si>
+    <t>IC MOTOR DRIVER 2V-5.2V 10VSSOP</t>
+  </si>
+  <si>
+    <t>TI</t>
+  </si>
+  <si>
+    <t>DRV2605LDGST</t>
+  </si>
+  <si>
+    <t>C425927</t>
+  </si>
+  <si>
     <t>BZ1, BZ2</t>
   </si>
   <si>
@@ -227,12 +278,6 @@
     <t>custombatteryconnector_small</t>
   </si>
   <si>
-    <t>C1, C2, C3, C4</t>
-  </si>
-  <si>
-    <t>FP-C0402-BB-MFG</t>
-  </si>
-  <si>
     <t>J3</t>
   </si>
   <si>
@@ -270,24 +315,6 @@
   </si>
   <si>
     <t>PROMICRO</t>
-  </si>
-  <si>
-    <t>U3, U5</t>
-  </si>
-  <si>
-    <t>FP-DGS0010A-MFG</t>
-  </si>
-  <si>
-    <t>IC MOTOR DRIVER 2V-5.2V 10VSSOP</t>
-  </si>
-  <si>
-    <t>U4, U6</t>
-  </si>
-  <si>
-    <t>SMD-16_ELV1411A</t>
-  </si>
-  <si>
-    <t>null</t>
   </si>
 </sst>
 </file>
@@ -683,7 +710,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98DFA7FA-7D81-43DF-9A76-31BD0DB688AC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{929C5415-AE39-43CB-8511-1C5FC016537F}">
   <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -743,7 +770,7 @@
         <v>14</v>
       </c>
       <c r="H2" s="1">
-        <v>42</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -769,7 +796,7 @@
         <v>20</v>
       </c>
       <c r="H3" s="1">
-        <v>2</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -786,33 +813,33 @@
         <v>24</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H4" s="1">
-        <v>42</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>13</v>
@@ -821,7 +848,7 @@
         <v>31</v>
       </c>
       <c r="H5" s="1">
-        <v>2</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -832,45 +859,45 @@
         <v>33</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H6" s="1">
-        <v>44</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H7" s="1">
         <v>2</v>
@@ -878,39 +905,39 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>48</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H8" s="1">
-        <v>2</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>52</v>
@@ -939,16 +966,16 @@
         <v>57</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H10" s="1">
         <v>2</v>
@@ -956,123 +983,147 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
+        <v>63</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="H11" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
+        <v>29</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="H12" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
+        <v>73</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>76</v>
+      </c>
       <c r="H13" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C14" s="1"/>
+        <v>78</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>10</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
-      <c r="F15" s="2" t="s">
-        <v>10</v>
-      </c>
+      <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>10</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
+      <c r="F17" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1">
         <v>2</v>
@@ -1080,31 +1131,31 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
@@ -1116,13 +1167,13 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>79</v>
+        <v>17</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
@@ -1134,21 +1185,17 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>82</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="D21" s="1"/>
       <c r="E21" s="1"/>
-      <c r="F21" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1">
         <v>2</v>

</xml_diff>

<commit_message>
fix haptic driver pos
</commit_message>
<xml_diff>
--- a/PCB/Altuim/Project Outputs for klor1_4/BOM/Bill of Materials-klor1_4.xlsx
+++ b/PCB/Altuim/Project Outputs for klor1_4/BOM/Bill of Materials-klor1_4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahmed\Work\KLOR\PCB\Altuim\Project Outputs for klor1_4\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF53B3FE-E58F-4809-89DF-E655BB02E827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A6117EF-4769-4752-92EF-3FA688098D06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{8F8EA070-2F4B-4877-A16D-FC4F2D8C15A9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1D02BBEF-149B-4C15-A048-0F2EF0ECAAF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-klor1_4" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
     <t>JLCPCB Assembly</t>
   </si>
   <si>
-    <t>ELV1411</t>
+    <t>ELV1411A</t>
   </si>
   <si>
     <t>LCSC</t>
@@ -710,7 +710,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{929C5415-AE39-43CB-8511-1C5FC016537F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6410257C-5953-405B-B9C9-4EFA56B92631}">
   <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>

<commit_message>
fixing NiceNano 3D orientation
</commit_message>
<xml_diff>
--- a/PCB/Altuim/Project Outputs for klor1_4/BOM/Bill of Materials-klor1_4.xlsx
+++ b/PCB/Altuim/Project Outputs for klor1_4/BOM/Bill of Materials-klor1_4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahmed\Work\KLOR\PCB\Altuim\Project Outputs for klor1_4\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A6117EF-4769-4752-92EF-3FA688098D06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DE3827E-287A-4ACB-BDAD-A1C7804A2821}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{1D02BBEF-149B-4C15-A048-0F2EF0ECAAF9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="82">
   <si>
     <t>Designator</t>
   </si>
@@ -272,49 +272,19 @@
     <t>C110293</t>
   </si>
   <si>
-    <t>BT2, BT4</t>
-  </si>
-  <si>
-    <t>custombatteryconnector_small</t>
-  </si>
-  <si>
-    <t>J3</t>
-  </si>
-  <si>
-    <t>lvc27_onlyInput</t>
-  </si>
-  <si>
-    <t>J5</t>
-  </si>
-  <si>
-    <t>JP26, JP29</t>
-  </si>
-  <si>
-    <t>SolderJumper-2_P1.3mm_Open_TrianglePad1.0x1.5mm</t>
-  </si>
-  <si>
-    <t>MH1, MH2, MH3, MH4, MH5, MH6, MH7, MH8, MH10, MH11, MH12, MH13, MH14, MH15, MH16, MH17</t>
-  </si>
-  <si>
-    <t>MOUNTINGHOLE_3.2MM_M3</t>
-  </si>
-  <si>
     <t>OLED1, OLED2</t>
   </si>
   <si>
     <t>SSD1306_128X64OLED</t>
   </si>
   <si>
-    <t>TP1, TP2</t>
-  </si>
-  <si>
-    <t>SplitkbTentingPuckWithoutCenterHole</t>
-  </si>
-  <si>
-    <t>U1, U2</t>
-  </si>
-  <si>
-    <t>PROMICRO</t>
+    <t>HS96L03W2C03</t>
+  </si>
+  <si>
+    <t>C5248080</t>
+  </si>
+  <si>
+    <t>HS</t>
   </si>
 </sst>
 </file>
@@ -711,7 +681,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6410257C-5953-405B-B9C9-4EFA56B92631}">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.81640625" customWidth="1"/>
@@ -1069,135 +1039,19 @@
       <c r="C14" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
+      <c r="D14" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>80</v>
+      </c>
       <c r="H14" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1">
         <v>2</v>
       </c>
     </row>

</xml_diff>